<commit_message>
Implemented all required models and compared with each and every model
</commit_message>
<xml_diff>
--- a/notebooks/JayaSaiKishore.xlsx
+++ b/notebooks/JayaSaiKishore.xlsx
@@ -413,494 +413,487 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A97"/>
+  <dimension ref="A1:A96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Power_KW</t>
-        </is>
+      <c r="A1" t="n">
+        <v>153.484234118501</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>150.9951844813046</v>
+        <v>152.6799530187779</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10.1592304753033</v>
+        <v>152.1711919220185</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>-0.790487764850802</v>
+        <v>152.3850777999161</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>11.67791005618442</v>
+        <v>152.7577512979187</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>11.67791005618442</v>
+        <v>151.0358784060245</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>11.43537976276933</v>
+        <v>148.8453989142415</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>11.43537976276933</v>
+        <v>151.1863478628754</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>11.43537976276933</v>
+        <v>149.55673722014</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11.43537976276933</v>
+        <v>151.1324247336399</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11.19284946935423</v>
+        <v>151.9474019664309</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11.19284946935423</v>
+        <v>152.0876033948745</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11.19284946935423</v>
+        <v>152.2590352435677</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>123.3828676575227</v>
+        <v>152.1998510750697</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>138.4868480575389</v>
+        <v>152.2420258952032</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>134.3931508417324</v>
+        <v>152.3771113960923</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>135.0279826124673</v>
+        <v>154.288112670768</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>142.6866587414893</v>
+        <v>153.796313504584</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>159.7470834058072</v>
+        <v>153.2051016940025</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>158.0960357324495</v>
+        <v>152.6305909704342</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>153.937098717865</v>
+        <v>152.9720154760949</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>140.7156025794318</v>
+        <v>154.4873981756267</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>151.6808045196576</v>
+        <v>154.1299621186186</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>159.4369536387519</v>
+        <v>153.2325769829377</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>155.547440140861</v>
+        <v>157.027008275524</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>152.4552492364418</v>
+        <v>161.0128476301579</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>161.86490843188</v>
+        <v>165.956905719026</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>157.3583185334083</v>
+        <v>170.765778580936</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>162.5477604648196</v>
+        <v>176.8350644125312</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>170.3668315870926</v>
+        <v>179.4959308565972</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>177.6291334780235</v>
+        <v>177.4227512070601</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>169.638832070542</v>
+        <v>172.6032517586278</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>152.2418696939955</v>
+        <v>173.7436476995422</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>155.631993746344</v>
+        <v>254.5310962559212</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>164.7706199539596</v>
+        <v>252.0860795899884</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>238.2135802406506</v>
+        <v>251.6717213336362</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>245.9114423430794</v>
+        <v>252.1044637202509</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>239.9086926628477</v>
+        <v>252.3469897410312</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>244.7676869756812</v>
+        <v>252.2480460131532</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>247.6129832568186</v>
+        <v>252.1502403182587</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>246.0097528014177</v>
+        <v>252.1645182798734</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>242.2654247146422</v>
+        <v>252.1664485176548</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>240.3406541131523</v>
+        <v>252.2129849729346</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>245.5722399004032</v>
+        <v>252.2227157468895</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>249.6678090807697</v>
+        <v>260.0850726353282</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>252.5602868717476</v>
+        <v>260.7361212656931</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>272.0949170594022</v>
+        <v>256.4791173380015</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>269.6767208395721</v>
+        <v>260.2963662325967</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>254.1846331421353</v>
+        <v>257.92215234127</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>279.8507618397551</v>
+        <v>260.8007711063145</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>254.7736221361003</v>
+        <v>261.9291801348996</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>266.1099776836827</v>
+        <v>258.8187210841789</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>279.650927338015</v>
+        <v>258.1816245045446</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>256.1086681507797</v>
+        <v>260.2396780416346</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>249.8632863933434</v>
+        <v>261.4935721348754</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>276.0719860614643</v>
+        <v>257.9794867522914</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>287.6693093511436</v>
+        <v>260.2020770062121</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>249.1815934960277</v>
+        <v>261.4365172441696</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>272.3742142156614</v>
+        <v>257.8938327401853</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>275.1725459830685</v>
+        <v>259.0474349249738</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>249.5062382348689</v>
+        <v>258.7433908485563</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>260.2741239550909</v>
+        <v>258.3590047555858</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>259.9595243784461</v>
+        <v>258.751648390747</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>259.6083468614486</v>
+        <v>258.2262181210367</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>262.352121782853</v>
+        <v>259.6932887950792</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>257.0018133960884</v>
+        <v>259.1388949820395</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>263.1376386538801</v>
+        <v>258.2114929043491</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>262.6839027331037</v>
+        <v>257.1065289665245</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>255.3238968226331</v>
+        <v>256.6781849370893</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>234.1744220395344</v>
+        <v>257.6242138047154</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>234.8509636161523</v>
+        <v>256.3395733350002</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>255.0137458033146</v>
+        <v>264.5958637194733</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>250.6100322017831</v>
+        <v>300.394097727273</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>275.5823275572719</v>
+        <v>298.1470282262508</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>305.4630505765005</v>
+        <v>300.2921579493272</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>292.1046021969622</v>
+        <v>298.1158094814748</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>298.2289994618195</v>
+        <v>298.3161270317653</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>296.6809871916007</v>
+        <v>300.3530437645286</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>297.050191373954</v>
+        <v>300.8579676408514</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>301.3448043012265</v>
+        <v>300.9416097003215</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>300.9612334165953</v>
+        <v>298.918861673914</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>300.4495963174315</v>
+        <v>298.1834039970386</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>296.9074118280242</v>
+        <v>293.4293742230063</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>296.4353754463981</v>
+        <v>293.2036411421481</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>285.1982380194974</v>
+        <v>292.5909026260256</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>283.220597741484</v>
+        <v>290.9505413688194</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>286.3489049383289</v>
+        <v>287.1350834561762</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>275.8655207984315</v>
+        <v>286.678739057697</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>270.4191086979126</v>
+        <v>284.6612235747527</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>272.9981492444533</v>
+        <v>283.6360466654912</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>268.2450089636854</v>
+        <v>282.4070440299909</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>271.836318792943</v>
+        <v>283.3822102029383</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>269.6514004260732</v>
+        <v>282.6187399645705</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>266.9284711284639</v>
+        <v>196.412299597666</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>267.3097641877525</v>
+        <v>194.2874749407404</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>200.4824247582888</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>185.0401750019249</v>
+        <v>160.3620431947837</v>
       </c>
     </row>
   </sheetData>

</xml_diff>